<commit_message>
datos: +151 sorteos hasta 2026-08-25
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2010" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2011" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2012" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2013" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2014" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2015" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2016" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2017" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2018" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2019" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2020" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2021" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2022" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2023" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2024" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="📊 Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2010" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2011" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2012" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2013" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2014" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2015" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2016" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2017" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2018" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2019" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2020" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2021" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2022" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="2023" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="2024" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="2025" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="2026" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,7 +34,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,6 +98,10 @@
       <name val="Calibri"/>
       <color rgb="00555555"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="18">
@@ -200,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -316,6 +320,7 @@
     <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -33415,7 +33420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B85"/>
+  <dimension ref="A1:B236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -34429,6 +34434,1818 @@
       <c r="A85" s="26" t="inlineStr">
         <is>
           <t>Total 2026: 82 sorteos  |  Generado 24/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="39" t="inlineStr">
+        <is>
+          <t>2026-03-25  Mié</t>
+        </is>
+      </c>
+      <c r="B86" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 09, 10, 15, 16, 25, 29, 33, 35, 39, 49, 52, 54, 58, 62, 63, 64, 71, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="39" t="inlineStr">
+        <is>
+          <t>2026-03-26  Jue</t>
+        </is>
+      </c>
+      <c r="B87" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 06, 14, 17, 18, 19, 22, 26, 28, 30, 33, 34, 42, 48, 51, 56, 59, 73, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="39" t="inlineStr">
+        <is>
+          <t>2026-03-27  Vie</t>
+        </is>
+      </c>
+      <c r="B88" s="39" t="inlineStr">
+        <is>
+          <t>14, 16, 17, 24, 25, 26, 27, 29, 45, 48, 49, 54, 60, 62, 64, 71, 73, 75, 78, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="39" t="inlineStr">
+        <is>
+          <t>2026-03-28  Sáb</t>
+        </is>
+      </c>
+      <c r="B89" s="39" t="inlineStr">
+        <is>
+          <t>04, 05, 06, 15, 17, 23, 27, 28, 32, 34, 36, 54, 60, 62, 63, 66, 68, 69, 75, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="39" t="inlineStr">
+        <is>
+          <t>2026-03-29  Dom</t>
+        </is>
+      </c>
+      <c r="B90" s="39" t="inlineStr">
+        <is>
+          <t>07, 18, 19, 21, 23, 29, 36, 37, 44, 48, 49, 50, 55, 59, 60, 66, 70, 71, 74, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="39" t="inlineStr">
+        <is>
+          <t>2026-03-30  Lun</t>
+        </is>
+      </c>
+      <c r="B91" s="39" t="inlineStr">
+        <is>
+          <t>01, 06, 09, 10, 13, 15, 19, 28, 30, 35, 37, 39, 42, 44, 45, 52, 59, 60, 64, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="39" t="inlineStr">
+        <is>
+          <t>2026-03-31  Mar</t>
+        </is>
+      </c>
+      <c r="B92" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 08, 10, 13, 25, 28, 31, 36, 40, 44, 49, 57, 59, 61, 64, 67, 72, 74, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-01  Mié</t>
+        </is>
+      </c>
+      <c r="B93" s="39" t="inlineStr">
+        <is>
+          <t>01, 04, 06, 07, 08, 09, 11, 26, 29, 39, 45, 46, 48, 49, 51, 54, 61, 63, 66, 67</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-04  Sáb</t>
+        </is>
+      </c>
+      <c r="B94" s="39" t="inlineStr">
+        <is>
+          <t>04, 05, 06, 10, 11, 12, 14, 21, 25, 28, 30, 33, 35, 37, 46, 53, 57, 65, 72, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-05  Dom</t>
+        </is>
+      </c>
+      <c r="B95" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 05, 09, 16, 20, 27, 29, 30, 31, 32, 33, 34, 36, 38, 40, 42, 43, 47, 51</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-06  Lun</t>
+        </is>
+      </c>
+      <c r="B96" s="39" t="inlineStr">
+        <is>
+          <t>03, 05, 06, 07, 08, 13, 14, 19, 27, 29, 32, 44, 45, 56, 63, 65, 73, 74, 76, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-07  Mar</t>
+        </is>
+      </c>
+      <c r="B97" s="39" t="inlineStr">
+        <is>
+          <t>01, 05, 07, 16, 17, 18, 22, 29, 31, 36, 43, 51, 54, 55, 60, 61, 64, 69, 71, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-08  Mié</t>
+        </is>
+      </c>
+      <c r="B98" s="39" t="inlineStr">
+        <is>
+          <t>05, 06, 07, 08, 09, 11, 13, 16, 21, 31, 34, 40, 41, 44, 47, 49, 53, 59, 61, 67</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-09  Jue</t>
+        </is>
+      </c>
+      <c r="B99" s="39" t="inlineStr">
+        <is>
+          <t>05, 08, 09, 13, 18, 21, 22, 30, 31, 41, 44, 47, 48, 53, 54, 59, 64, 65, 67, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-10  Vie</t>
+        </is>
+      </c>
+      <c r="B100" s="39" t="inlineStr">
+        <is>
+          <t>07, 10, 26, 33, 36, 38, 41, 44, 51, 52, 54, 55, 56, 60, 63, 64, 66, 67, 72, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-11  Sáb</t>
+        </is>
+      </c>
+      <c r="B101" s="39" t="inlineStr">
+        <is>
+          <t>08, 11, 13, 15, 20, 25, 28, 31, 32, 35, 43, 44, 46, 48, 54, 66, 70, 71, 74, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-12  Dom</t>
+        </is>
+      </c>
+      <c r="B102" s="39" t="inlineStr">
+        <is>
+          <t>12, 13, 14, 16, 21, 29, 34, 41, 51, 53, 54, 55, 56, 61, 62, 68, 70, 73, 74, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-13  Lun</t>
+        </is>
+      </c>
+      <c r="B103" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 05, 10, 11, 13, 14, 17, 23, 25, 31, 34, 47, 51, 53, 61, 70, 71, 72, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-14  Mar</t>
+        </is>
+      </c>
+      <c r="B104" s="39" t="inlineStr">
+        <is>
+          <t>05, 06, 14, 23, 28, 30, 31, 34, 44, 49, 52, 56, 57, 58, 63, 66, 67, 68, 74, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-15  Mié</t>
+        </is>
+      </c>
+      <c r="B105" s="39" t="inlineStr">
+        <is>
+          <t>02, 06, 12, 15, 19, 23, 24, 35, 37, 38, 39, 40, 41, 47, 58, 59, 64, 67, 68, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-16  Jue</t>
+        </is>
+      </c>
+      <c r="B106" s="39" t="inlineStr">
+        <is>
+          <t>03, 06, 11, 13, 15, 16, 18, 25, 32, 33, 35, 42, 44, 49, 51, 54, 59, 61, 63, 67</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-17  Vie</t>
+        </is>
+      </c>
+      <c r="B107" s="39" t="inlineStr">
+        <is>
+          <t>01, 04, 10, 17, 33, 35, 37, 40, 44, 46, 49, 50, 51, 52, 54, 56, 59, 62, 70, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-18  Sáb</t>
+        </is>
+      </c>
+      <c r="B108" s="39" t="inlineStr">
+        <is>
+          <t>03, 12, 14, 15, 18, 22, 32, 34, 35, 42, 46, 48, 55, 56, 58, 61, 62, 66, 74, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-19  Dom</t>
+        </is>
+      </c>
+      <c r="B109" s="39" t="inlineStr">
+        <is>
+          <t>03, 04, 05, 07, 08, 13, 14, 19, 25, 38, 50, 51, 52, 57, 58, 62, 71, 73, 74, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-20  Lun</t>
+        </is>
+      </c>
+      <c r="B110" s="39" t="inlineStr">
+        <is>
+          <t>02, 05, 06, 07, 08, 12, 14, 18, 20, 21, 24, 26, 36, 44, 52, 55, 58, 59, 70, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-21  Mar</t>
+        </is>
+      </c>
+      <c r="B111" s="39" t="inlineStr">
+        <is>
+          <t>01, 05, 06, 14, 21, 30, 34, 40, 42, 43, 44, 46, 48, 52, 55, 61, 67, 69, 73, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-22  Mié</t>
+        </is>
+      </c>
+      <c r="B112" s="39" t="inlineStr">
+        <is>
+          <t>07, 10, 13, 19, 20, 21, 22, 25, 28, 29, 30, 36, 40, 45, 47, 48, 54, 62, 75, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-23  Jue</t>
+        </is>
+      </c>
+      <c r="B113" s="39" t="inlineStr">
+        <is>
+          <t>05, 12, 16, 17, 21, 23, 25, 29, 30, 34, 38, 42, 43, 46, 50, 56, 57, 61, 68, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-24  Vie</t>
+        </is>
+      </c>
+      <c r="B114" s="39" t="inlineStr">
+        <is>
+          <t>01, 04, 10, 12, 15, 19, 24, 25, 26, 28, 30, 31, 34, 38, 39, 46, 60, 62, 67, 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-25  Sáb</t>
+        </is>
+      </c>
+      <c r="B115" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 14, 18, 23, 25, 28, 38, 39, 44, 47, 49, 51, 52, 59, 64, 66, 72, 74, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-26  Dom</t>
+        </is>
+      </c>
+      <c r="B116" s="39" t="inlineStr">
+        <is>
+          <t>01, 10, 12, 13, 16, 22, 23, 25, 26, 29, 33, 37, 43, 44, 50, 52, 58, 63, 69, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-27  Lun</t>
+        </is>
+      </c>
+      <c r="B117" s="39" t="inlineStr">
+        <is>
+          <t>04, 06, 07, 10, 16, 18, 23, 26, 27, 33, 35, 37, 39, 45, 48, 55, 56, 58, 65, 66</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-28  Mar</t>
+        </is>
+      </c>
+      <c r="B118" s="39" t="inlineStr">
+        <is>
+          <t>08, 10, 12, 14, 20, 23, 24, 28, 34, 37, 39, 41, 42, 43, 46, 47, 48, 55, 63, 67</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-29  Mié</t>
+        </is>
+      </c>
+      <c r="B119" s="39" t="inlineStr">
+        <is>
+          <t>01, 05, 08, 09, 13, 15, 17, 20, 24, 29, 30, 32, 34, 35, 37, 43, 48, 52, 60, 64</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="39" t="inlineStr">
+        <is>
+          <t>2026-04-30  Jue</t>
+        </is>
+      </c>
+      <c r="B120" s="39" t="inlineStr">
+        <is>
+          <t>05, 10, 12, 13, 14, 15, 30, 31, 33, 34, 36, 48, 50, 55, 59, 61, 68, 69, 71, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-01  Vie</t>
+        </is>
+      </c>
+      <c r="B121" s="39" t="inlineStr">
+        <is>
+          <t>01, 10, 12, 16, 18, 23, 27, 29, 36, 37, 39, 42, 43, 46, 50, 54, 59, 63, 71, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-02  Sáb</t>
+        </is>
+      </c>
+      <c r="B122" s="39" t="inlineStr">
+        <is>
+          <t>02, 07, 11, 14, 22, 23, 29, 34, 35, 37, 39, 42, 43, 44, 47, 52, 55, 56, 63, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-03  Dom</t>
+        </is>
+      </c>
+      <c r="B123" s="39" t="inlineStr">
+        <is>
+          <t>03, 07, 08, 15, 20, 21, 22, 23, 37, 38, 40, 42, 48, 49, 52, 59, 63, 65, 67, 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-04  Lun</t>
+        </is>
+      </c>
+      <c r="B124" s="39" t="inlineStr">
+        <is>
+          <t>04, 09, 10, 17, 24, 30, 32, 40, 47, 51, 53, 54, 61, 63, 65, 66, 67, 75, 76, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-05  Mar</t>
+        </is>
+      </c>
+      <c r="B125" s="39" t="inlineStr">
+        <is>
+          <t>02, 05, 07, 14, 15, 24, 31, 33, 38, 39, 40, 42, 50, 51, 55, 57, 58, 59, 63, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-06  Mié</t>
+        </is>
+      </c>
+      <c r="B126" s="39" t="inlineStr">
+        <is>
+          <t>04, 06, 07, 10, 15, 16, 17, 18, 20, 25, 32, 38, 40, 45, 51, 63, 64, 65, 69, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-07  Jue</t>
+        </is>
+      </c>
+      <c r="B127" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 07, 11, 13, 14, 15, 17, 24, 25, 34, 39, 43, 46, 50, 59, 62, 64, 70, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-08  Vie</t>
+        </is>
+      </c>
+      <c r="B128" s="39" t="inlineStr">
+        <is>
+          <t>08, 13, 14, 15, 16, 21, 28, 31, 32, 40, 46, 49, 50, 53, 54, 59, 64, 66, 70, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-09  Sáb</t>
+        </is>
+      </c>
+      <c r="B129" s="39" t="inlineStr">
+        <is>
+          <t>03, 07, 08, 09, 14, 15, 21, 33, 34, 43, 49, 51, 63, 64, 66, 68, 71, 74, 76, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-10  Dom</t>
+        </is>
+      </c>
+      <c r="B130" s="39" t="inlineStr">
+        <is>
+          <t>04, 06, 10, 17, 21, 23, 29, 32, 35, 39, 40, 43, 45, 47, 48, 52, 65, 69, 72, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-11  Lun</t>
+        </is>
+      </c>
+      <c r="B131" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 11, 12, 17, 19, 29, 34, 39, 41, 42, 44, 46, 50, 54, 58, 61, 64, 69, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-12  Mar</t>
+        </is>
+      </c>
+      <c r="B132" s="39" t="inlineStr">
+        <is>
+          <t>05, 12, 26, 27, 28, 30, 32, 36, 42, 46, 49, 50, 56, 57, 59, 63, 65, 70, 72, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-13  Mié</t>
+        </is>
+      </c>
+      <c r="B133" s="39" t="inlineStr">
+        <is>
+          <t>11, 13, 15, 16, 23, 26, 27, 29, 35, 36, 41, 46, 47, 48, 54, 56, 58, 59, 67, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-14  Jue</t>
+        </is>
+      </c>
+      <c r="B134" s="39" t="inlineStr">
+        <is>
+          <t>03, 05, 14, 15, 20, 23, 26, 30, 39, 42, 43, 47, 51, 52, 61, 62, 63, 65, 67, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-15  Vie</t>
+        </is>
+      </c>
+      <c r="B135" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 05, 12, 15, 18, 36, 37, 43, 44, 50, 53, 56, 57, 60, 63, 66, 70, 71, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-16  Sáb</t>
+        </is>
+      </c>
+      <c r="B136" s="39" t="inlineStr">
+        <is>
+          <t>02, 05, 09, 16, 29, 31, 33, 36, 40, 41, 42, 45, 47, 49, 54, 55, 60, 70, 71, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-17  Dom</t>
+        </is>
+      </c>
+      <c r="B137" s="39" t="inlineStr">
+        <is>
+          <t>03, 15, 17, 19, 23, 26, 27, 31, 32, 36, 39, 48, 51, 52, 56, 60, 63, 68, 71, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-18  Lun</t>
+        </is>
+      </c>
+      <c r="B138" s="39" t="inlineStr">
+        <is>
+          <t>06, 12, 14, 17, 18, 26, 32, 33, 36, 44, 52, 56, 59, 60, 61, 64, 65, 68, 76, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-19  Mar</t>
+        </is>
+      </c>
+      <c r="B139" s="39" t="inlineStr">
+        <is>
+          <t>07, 08, 11, 16, 17, 19, 22, 23, 24, 28, 37, 39, 46, 47, 61, 63, 65, 66, 68, 71</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-20  Mié</t>
+        </is>
+      </c>
+      <c r="B140" s="39" t="inlineStr">
+        <is>
+          <t>03, 05, 09, 12, 13, 20, 21, 26, 27, 33, 35, 40, 41, 45, 56, 61, 63, 64, 68, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-21  Jue</t>
+        </is>
+      </c>
+      <c r="B141" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 07, 08, 14, 21, 23, 25, 27, 28, 35, 37, 40, 43, 46, 47, 56, 57, 76, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-22  Vie</t>
+        </is>
+      </c>
+      <c r="B142" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 11, 18, 22, 25, 29, 30, 32, 34, 39, 41, 42, 46, 52, 54, 55, 57, 59, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-23  Sáb</t>
+        </is>
+      </c>
+      <c r="B143" s="39" t="inlineStr">
+        <is>
+          <t>01, 07, 09, 11, 14, 18, 20, 21, 23, 24, 25, 29, 32, 38, 51, 55, 57, 59, 75, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-24  Dom</t>
+        </is>
+      </c>
+      <c r="B144" s="39" t="inlineStr">
+        <is>
+          <t>01, 04, 08, 16, 17, 19, 21, 23, 24, 26, 27, 29, 34, 51, 55, 61, 62, 66, 68, 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-25  Lun</t>
+        </is>
+      </c>
+      <c r="B145" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 07, 10, 13, 15, 17, 22, 23, 25, 37, 41, 44, 46, 50, 60, 65, 67, 73, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-26  Mar</t>
+        </is>
+      </c>
+      <c r="B146" s="39" t="inlineStr">
+        <is>
+          <t>02, 06, 07, 09, 14, 19, 20, 21, 24, 26, 28, 36, 38, 47, 52, 54, 60, 61, 63, 65</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-27  Mié</t>
+        </is>
+      </c>
+      <c r="B147" s="39" t="inlineStr">
+        <is>
+          <t>03, 04, 05, 06, 18, 19, 27, 28, 34, 36, 37, 43, 45, 46, 55, 57, 58, 65, 69, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-28  Jue</t>
+        </is>
+      </c>
+      <c r="B148" s="39" t="inlineStr">
+        <is>
+          <t>08, 11, 19, 24, 28, 30, 31, 32, 33, 41, 42, 48, 54, 57, 60, 61, 63, 71, 72, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-29  Vie</t>
+        </is>
+      </c>
+      <c r="B149" s="39" t="inlineStr">
+        <is>
+          <t>04, 06, 07, 11, 18, 23, 26, 29, 37, 39, 41, 42, 51, 52, 55, 64, 66, 74, 76, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-30  Sáb</t>
+        </is>
+      </c>
+      <c r="B150" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 09, 20, 24, 25, 26, 28, 30, 31, 35, 36, 50, 52, 55, 58, 63, 66, 73, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="39" t="inlineStr">
+        <is>
+          <t>2026-05-31  Dom</t>
+        </is>
+      </c>
+      <c r="B151" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 06, 09, 10, 13, 16, 17, 20, 25, 30, 31, 37, 38, 39, 40, 44, 49, 50, 55</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-01  Lun</t>
+        </is>
+      </c>
+      <c r="B152" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 03, 10, 12, 14, 15, 17, 27, 37, 40, 51, 55, 57, 59, 61, 63, 69, 74, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-02  Mar</t>
+        </is>
+      </c>
+      <c r="B153" s="39" t="inlineStr">
+        <is>
+          <t>02, 08, 10, 12, 16, 18, 19, 23, 27, 28, 33, 40, 43, 46, 65, 67, 68, 71, 72, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-03  Mié</t>
+        </is>
+      </c>
+      <c r="B154" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 07, 11, 19, 32, 34, 35, 37, 38, 44, 46, 49, 51, 52, 53, 55, 59, 67, 71</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-04  Jue</t>
+        </is>
+      </c>
+      <c r="B155" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 05, 07, 12, 16, 27, 37, 40, 41, 44, 50, 55, 56, 60, 61, 63, 65, 66, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-05  Vie</t>
+        </is>
+      </c>
+      <c r="B156" s="39" t="inlineStr">
+        <is>
+          <t>03, 05, 07, 08, 11, 12, 23, 24, 31, 33, 42, 47, 55, 59, 70, 71, 73, 74, 76, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-06  Sáb</t>
+        </is>
+      </c>
+      <c r="B157" s="39" t="inlineStr">
+        <is>
+          <t>03, 06, 07, 12, 24, 28, 36, 39, 40, 45, 49, 60, 62, 64, 67, 75, 77, 78, 79, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-07  Dom</t>
+        </is>
+      </c>
+      <c r="B158" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 04, 06, 07, 09, 10, 14, 16, 17, 24, 30, 35, 49, 52, 54, 62, 72, 74, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-08  Lun</t>
+        </is>
+      </c>
+      <c r="B159" s="39" t="inlineStr">
+        <is>
+          <t>03, 08, 14, 16, 19, 23, 26, 32, 33, 37, 42, 45, 52, 56, 64, 65, 67, 69, 71, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-09  Mar</t>
+        </is>
+      </c>
+      <c r="B160" s="39" t="inlineStr">
+        <is>
+          <t>03, 04, 07, 09, 12, 14, 18, 20, 25, 33, 40, 41, 44, 55, 56, 57, 64, 68, 72, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-10  Mié</t>
+        </is>
+      </c>
+      <c r="B161" s="39" t="inlineStr">
+        <is>
+          <t>03, 10, 16, 20, 23, 30, 34, 37, 39, 40, 41, 46, 50, 51, 52, 57, 60, 63, 70, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-11  Jue</t>
+        </is>
+      </c>
+      <c r="B162" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 09, 11, 14, 17, 18, 20, 23, 31, 32, 34, 38, 40, 42, 46, 53, 58, 60, 64</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-12  Vie</t>
+        </is>
+      </c>
+      <c r="B163" s="39" t="inlineStr">
+        <is>
+          <t>12, 24, 25, 27, 38, 39, 44, 45, 50, 52, 56, 57, 61, 63, 64, 66, 72, 74, 75, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-13  Sáb</t>
+        </is>
+      </c>
+      <c r="B164" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 03, 13, 15, 16, 17, 19, 21, 23, 24, 25, 33, 37, 38, 50, 55, 59, 60, 61</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-14  Dom</t>
+        </is>
+      </c>
+      <c r="B165" s="39" t="inlineStr">
+        <is>
+          <t>02, 08, 09, 14, 16, 23, 24, 25, 28, 32, 34, 35, 38, 53, 55, 57, 64, 65, 68, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-15  Lun</t>
+        </is>
+      </c>
+      <c r="B166" s="39" t="inlineStr">
+        <is>
+          <t>05, 06, 15, 17, 21, 25, 26, 28, 30, 37, 41, 43, 46, 48, 50, 52, 61, 73, 78, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-16  Mar</t>
+        </is>
+      </c>
+      <c r="B167" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 09, 11, 13, 16, 17, 22, 23, 24, 32, 39, 42, 43, 48, 50, 51, 53, 62, 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-17  Mié</t>
+        </is>
+      </c>
+      <c r="B168" s="39" t="inlineStr">
+        <is>
+          <t>07, 10, 11, 13, 17, 18, 19, 25, 26, 28, 30, 31, 37, 43, 61, 62, 69, 71, 73, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-18  Jue</t>
+        </is>
+      </c>
+      <c r="B169" s="39" t="inlineStr">
+        <is>
+          <t>06, 08, 10, 12, 15, 16, 17, 18, 34, 35, 43, 45, 49, 54, 56, 57, 58, 60, 62, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-19  Vie</t>
+        </is>
+      </c>
+      <c r="B170" s="39" t="inlineStr">
+        <is>
+          <t>05, 17, 19, 22, 31, 33, 35, 43, 46, 47, 53, 55, 56, 59, 61, 63, 69, 71, 72, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-20  Sáb</t>
+        </is>
+      </c>
+      <c r="B171" s="39" t="inlineStr">
+        <is>
+          <t>03, 05, 07, 12, 13, 19, 20, 21, 25, 27, 29, 32, 36, 41, 45, 46, 47, 52, 55, 63</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-21  Dom</t>
+        </is>
+      </c>
+      <c r="B172" s="39" t="inlineStr">
+        <is>
+          <t>05, 08, 09, 15, 18, 21, 23, 24, 25, 27, 32, 36, 37, 39, 47, 49, 55, 58, 68, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-22  Lun</t>
+        </is>
+      </c>
+      <c r="B173" s="39" t="inlineStr">
+        <is>
+          <t>18, 21, 22, 25, 26, 28, 32, 33, 34, 35, 37, 39, 41, 42, 45, 48, 50, 56, 57, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-24  Mié</t>
+        </is>
+      </c>
+      <c r="B174" s="39" t="inlineStr">
+        <is>
+          <t>11, 13, 18, 23, 24, 31, 33, 39, 46, 48, 51, 56, 59, 60, 64, 66, 68, 73, 76, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-25  Jue</t>
+        </is>
+      </c>
+      <c r="B175" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 05, 07, 12, 13, 19, 20, 25, 28, 29, 31, 35, 40, 44, 50, 52, 60, 63, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-26  Vie</t>
+        </is>
+      </c>
+      <c r="B176" s="39" t="inlineStr">
+        <is>
+          <t>02, 05, 18, 20, 23, 26, 27, 32, 34, 46, 55, 56, 59, 61, 63, 69, 73, 76, 79, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-27  Sáb</t>
+        </is>
+      </c>
+      <c r="B177" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 05, 10, 13, 19, 21, 27, 34, 35, 40, 47, 48, 50, 52, 64, 70, 74, 77, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-28  Dom</t>
+        </is>
+      </c>
+      <c r="B178" s="39" t="inlineStr">
+        <is>
+          <t>06, 11, 17, 21, 27, 28, 35, 38, 41, 43, 46, 48, 57, 60, 63, 64, 66, 69, 72, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-29  Lun</t>
+        </is>
+      </c>
+      <c r="B179" s="39" t="inlineStr">
+        <is>
+          <t>01, 07, 08, 12, 13, 14, 22, 23, 26, 29, 31, 40, 42, 51, 52, 53, 55, 67, 68, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="39" t="inlineStr">
+        <is>
+          <t>2026-06-30  Mar</t>
+        </is>
+      </c>
+      <c r="B180" s="39" t="inlineStr">
+        <is>
+          <t>05, 07, 11, 14, 15, 23, 24, 29, 30, 33, 35, 43, 44, 48, 55, 59, 61, 63, 70, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-01  Mié</t>
+        </is>
+      </c>
+      <c r="B181" s="39" t="inlineStr">
+        <is>
+          <t>01, 14, 19, 25, 27, 28, 37, 39, 42, 47, 51, 52, 57, 58, 60, 65, 72, 73, 76, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-02  Jue</t>
+        </is>
+      </c>
+      <c r="B182" s="39" t="inlineStr">
+        <is>
+          <t>02, 05, 14, 22, 25, 28, 29, 35, 37, 38, 42, 45, 46, 58, 61, 65, 67, 69, 73, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-03  Vie</t>
+        </is>
+      </c>
+      <c r="B183" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 04, 08, 16, 26, 32, 34, 38, 39, 40, 41, 44, 58, 59, 64, 68, 74, 76, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-04  Sáb</t>
+        </is>
+      </c>
+      <c r="B184" s="39" t="inlineStr">
+        <is>
+          <t>01, 04, 06, 10, 11, 17, 19, 20, 21, 32, 33, 39, 40, 43, 55, 57, 62, 71, 76, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-05  Dom</t>
+        </is>
+      </c>
+      <c r="B185" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 05, 12, 14, 23, 29, 33, 35, 37, 38, 45, 49, 50, 53, 55, 59, 60, 63, 67</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-06  Lun</t>
+        </is>
+      </c>
+      <c r="B186" s="39" t="inlineStr">
+        <is>
+          <t>02, 06, 09, 14, 16, 17, 29, 33, 39, 40, 42, 56, 58, 59, 60, 64, 68, 73, 77, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-07  Mar</t>
+        </is>
+      </c>
+      <c r="B187" s="39" t="inlineStr">
+        <is>
+          <t>07, 10, 17, 23, 24, 26, 28, 29, 43, 44, 47, 50, 53, 54, 57, 59, 60, 63, 71, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-08  Mié</t>
+        </is>
+      </c>
+      <c r="B188" s="39" t="inlineStr">
+        <is>
+          <t>08, 10, 17, 23, 24, 26, 28, 29, 43, 44, 47, 50, 53, 54, 57, 59, 60, 63, 71, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-09  Jue</t>
+        </is>
+      </c>
+      <c r="B189" s="39" t="inlineStr">
+        <is>
+          <t>01, 05, 07, 09, 10, 15, 25, 28, 32, 35, 43, 49, 50, 52, 53, 61, 64, 65, 66, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-10  Vie</t>
+        </is>
+      </c>
+      <c r="B190" s="39" t="inlineStr">
+        <is>
+          <t>01, 05, 07, 10, 14, 18, 24, 25, 33, 35, 41, 54, 55, 58, 63, 64, 68, 73, 78, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-11  Sáb</t>
+        </is>
+      </c>
+      <c r="B191" s="39" t="inlineStr">
+        <is>
+          <t>01, 05, 11, 12, 24, 25, 28, 29, 31, 33, 34, 35, 36, 39, 43, 45, 50, 51, 53, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-12  Dom</t>
+        </is>
+      </c>
+      <c r="B192" s="39" t="inlineStr">
+        <is>
+          <t>03, 09, 12, 14, 21, 22, 23, 28, 41, 45, 48, 50, 51, 53, 54, 57, 58, 61, 69, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-13  Lun</t>
+        </is>
+      </c>
+      <c r="B193" s="39" t="inlineStr">
+        <is>
+          <t>02, 06, 08, 13, 16, 17, 25, 26, 28, 30, 33, 44, 51, 57, 59, 66, 69, 74, 76, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-14  Mar</t>
+        </is>
+      </c>
+      <c r="B194" s="39" t="inlineStr">
+        <is>
+          <t>14, 16, 19, 21, 23, 26, 40, 45, 46, 49, 56, 60, 65, 67, 69, 70, 71, 77, 78, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-15  Mié</t>
+        </is>
+      </c>
+      <c r="B195" s="39" t="inlineStr">
+        <is>
+          <t>03, 08, 11, 15, 16, 18, 25, 33, 41, 44, 50, 51, 57, 58, 60, 69, 70, 72, 74, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-16  Jue</t>
+        </is>
+      </c>
+      <c r="B196" s="39" t="inlineStr">
+        <is>
+          <t>04, 10, 11, 12, 16, 18, 30, 38, 40, 42, 44, 46, 48, 53, 56, 61, 62, 64, 77, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-17  Vie</t>
+        </is>
+      </c>
+      <c r="B197" s="39" t="inlineStr">
+        <is>
+          <t>07, 11, 13, 16, 17, 19, 21, 22, 28, 29, 31, 32, 35, 44, 45, 46, 57, 59, 67, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-18  Sáb</t>
+        </is>
+      </c>
+      <c r="B198" s="39" t="inlineStr">
+        <is>
+          <t>03, 06, 12, 14, 18, 20, 26, 36, 37, 40, 43, 44, 45, 46, 50, 54, 56, 61, 65, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-19  Dom</t>
+        </is>
+      </c>
+      <c r="B199" s="39" t="inlineStr">
+        <is>
+          <t>03, 06, 16, 19, 24, 26, 30, 46, 48, 51, 52, 62, 67, 68, 71, 72, 73, 74, 76, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-20  Lun</t>
+        </is>
+      </c>
+      <c r="B200" s="39" t="inlineStr">
+        <is>
+          <t>01, 06, 07, 13, 14, 17, 19, 20, 24, 29, 30, 36, 52, 59, 62, 63, 66, 67, 74, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-21  Mar</t>
+        </is>
+      </c>
+      <c r="B201" s="39" t="inlineStr">
+        <is>
+          <t>02, 07, 08, 10, 19, 21, 22, 29, 32, 33, 37, 38, 40, 43, 45, 49, 55, 56, 65, 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-22  Mié</t>
+        </is>
+      </c>
+      <c r="B202" s="39" t="inlineStr">
+        <is>
+          <t>03, 04, 05, 06, 13, 14, 20, 22, 29, 30, 32, 33, 34, 40, 50, 60, 63, 64, 66, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-23  Jue</t>
+        </is>
+      </c>
+      <c r="B203" s="39" t="inlineStr">
+        <is>
+          <t>06, 08, 11, 13, 18, 20, 23, 28, 35, 40, 41, 43, 44, 48, 53, 56, 59, 68, 69, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-24  Vie</t>
+        </is>
+      </c>
+      <c r="B204" s="39" t="inlineStr">
+        <is>
+          <t>02, 09, 10, 11, 13, 14, 19, 23, 24, 25, 27, 49, 50, 51, 57, 59, 61, 65, 71, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-25  Sáb</t>
+        </is>
+      </c>
+      <c r="B205" s="39" t="inlineStr">
+        <is>
+          <t>01, 06, 08, 12, 15, 18, 21, 25, 31, 38, 39, 50, 53, 58, 62, 66, 72, 73, 75, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-26  Dom</t>
+        </is>
+      </c>
+      <c r="B206" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 05, 06, 07, 09, 12, 16, 18, 23, 26, 27, 33, 35, 44, 46, 66, 67, 76, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-27  Lun</t>
+        </is>
+      </c>
+      <c r="B207" s="39" t="inlineStr">
+        <is>
+          <t>08, 10, 11, 12, 21, 23, 27, 32, 36, 38, 44, 49, 52, 56, 60, 61, 62, 65, 67, 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-28  Mar</t>
+        </is>
+      </c>
+      <c r="B208" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 06, 14, 17, 18, 26, 28, 35, 36, 42, 44, 45, 47, 50, 53, 69, 73, 78, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-29  Mié</t>
+        </is>
+      </c>
+      <c r="B209" s="39" t="inlineStr">
+        <is>
+          <t>07, 10, 11, 14, 21, 22, 29, 30, 32, 33, 34, 45, 48, 49, 51, 56, 57, 63, 65, 66</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-30  Jue</t>
+        </is>
+      </c>
+      <c r="B210" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 04, 07, 08, 10, 21, 26, 29, 30, 34, 36, 37, 58, 61, 68, 70, 71, 77, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-31  Vie</t>
+        </is>
+      </c>
+      <c r="B211" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 04, 05, 12, 14, 17, 26, 27, 30, 31, 35, 47, 49, 58, 59, 60, 66, 69, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-01  Sáb</t>
+        </is>
+      </c>
+      <c r="B212" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 04, 08, 28, 29, 35, 36, 40, 49, 51, 58, 59, 61, 65, 68, 71, 73, 74, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-02  Dom</t>
+        </is>
+      </c>
+      <c r="B213" s="39" t="inlineStr">
+        <is>
+          <t>02, 06, 13, 19, 21, 22, 29, 34, 36, 37, 38, 39, 40, 41, 43, 45, 48, 57, 60, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-03  Lun</t>
+        </is>
+      </c>
+      <c r="B214" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 06, 10, 14, 18, 20, 28, 32, 34, 35, 39, 40, 44, 58, 59, 60, 67, 75, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-04  Mar</t>
+        </is>
+      </c>
+      <c r="B215" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 11, 12, 14, 26, 27, 30, 36, 37, 40, 44, 53, 55, 57, 58, 63, 69, 72, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-05  Mié</t>
+        </is>
+      </c>
+      <c r="B216" s="39" t="inlineStr">
+        <is>
+          <t>05, 11, 13, 16, 17, 19, 25, 27, 32, 33, 35, 38, 40, 44, 52, 55, 58, 59, 62, 63</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-06  Jue</t>
+        </is>
+      </c>
+      <c r="B217" s="39" t="inlineStr">
+        <is>
+          <t>02, 05, 06, 09, 10, 16, 25, 26, 40, 41, 44, 47, 48, 49, 52, 59, 61, 65, 70, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-07  Vie</t>
+        </is>
+      </c>
+      <c r="B218" s="39" t="inlineStr">
+        <is>
+          <t>04, 07, 12, 18, 19, 26, 30, 38, 41, 42, 43, 47, 48, 50, 51, 52, 58, 62, 71, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-08  Sáb</t>
+        </is>
+      </c>
+      <c r="B219" s="39" t="inlineStr">
+        <is>
+          <t>01, 08, 09, 13, 18, 21, 31, 34, 36, 39, 40, 41, 42, 43, 44, 49, 50, 58, 69, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-09  Dom</t>
+        </is>
+      </c>
+      <c r="B220" s="39" t="inlineStr">
+        <is>
+          <t>03, 06, 08, 09, 14, 19, 21, 22, 27, 28, 30, 31, 34, 41, 44, 49, 50, 55, 57, 59</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-10  Lun</t>
+        </is>
+      </c>
+      <c r="B221" s="39" t="inlineStr">
+        <is>
+          <t>01, 10, 13, 22, 23, 24, 25, 31, 32, 37, 39, 48, 49, 51, 54, 55, 65, 66, 67, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-11  Mar</t>
+        </is>
+      </c>
+      <c r="B222" s="39" t="inlineStr">
+        <is>
+          <t>06, 11, 16, 20, 22, 24, 25, 35, 40, 41, 45, 50, 58, 61, 62, 63, 66, 73, 75, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-12  Mié</t>
+        </is>
+      </c>
+      <c r="B223" s="39" t="inlineStr">
+        <is>
+          <t>04, 10, 12, 13, 14, 17, 19, 22, 23, 26, 28, 36, 46, 52, 56, 62, 64, 67, 72, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-13  Jue</t>
+        </is>
+      </c>
+      <c r="B224" s="39" t="inlineStr">
+        <is>
+          <t>05, 06, 07, 11, 13, 14, 31, 33, 34, 37, 38, 43, 45, 50, 51, 62, 65, 68, 73, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-14  Vie</t>
+        </is>
+      </c>
+      <c r="B225" s="39" t="inlineStr">
+        <is>
+          <t>10, 11, 14, 16, 18, 25, 26, 28, 35, 41, 52, 56, 57, 58, 68, 69, 70, 71, 78, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-15  Sáb</t>
+        </is>
+      </c>
+      <c r="B226" s="39" t="inlineStr">
+        <is>
+          <t>02, 05, 13, 14, 15, 16, 19, 23, 25, 41, 50, 51, 58, 62, 66, 69, 73, 75, 77, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-16  Dom</t>
+        </is>
+      </c>
+      <c r="B227" s="39" t="inlineStr">
+        <is>
+          <t>08, 16, 21, 24, 30, 32, 33, 40, 42, 47, 50, 56, 62, 63, 64, 68, 71, 72, 77, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-17  Lun</t>
+        </is>
+      </c>
+      <c r="B228" s="39" t="inlineStr">
+        <is>
+          <t>05, 17, 18, 19, 21, 22, 23, 30, 32, 37, 39, 40, 42, 50, 53, 55, 68, 71, 73, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-18  Mar</t>
+        </is>
+      </c>
+      <c r="B229" s="39" t="inlineStr">
+        <is>
+          <t>12, 13, 17, 18, 20, 22, 23, 25, 27, 37, 39, 42, 46, 48, 57, 65, 70, 72, 74, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-19  Mié</t>
+        </is>
+      </c>
+      <c r="B230" s="39" t="inlineStr">
+        <is>
+          <t>02, 10, 13, 15, 19, 26, 33, 36, 37, 44, 45, 49, 52, 56, 57, 58, 59, 62, 63, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-20  Jue</t>
+        </is>
+      </c>
+      <c r="B231" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 07, 12, 15, 20, 23, 27, 30, 37, 38, 42, 43, 50, 55, 56, 59, 71, 72, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-21  Vie</t>
+        </is>
+      </c>
+      <c r="B232" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 04, 07, 18, 21, 23, 24, 26, 32, 39, 40, 44, 50, 54, 56, 61, 64, 67, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-22  Sáb</t>
+        </is>
+      </c>
+      <c r="B233" s="39" t="inlineStr">
+        <is>
+          <t>03, 07, 21, 22, 25, 26, 27, 28, 38, 39, 40, 47, 48, 51, 52, 58, 62, 65, 70, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-23  Dom</t>
+        </is>
+      </c>
+      <c r="B234" s="39" t="inlineStr">
+        <is>
+          <t>03, 04, 06, 07, 11, 12, 13, 19, 22, 23, 25, 32, 33, 37, 40, 49, 52, 56, 68, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-24  Lun</t>
+        </is>
+      </c>
+      <c r="B235" s="39" t="inlineStr">
+        <is>
+          <t>02, 05, 07, 08, 12, 14, 15, 17, 20, 22, 24, 27, 29, 37, 55, 56, 57, 60, 64, 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-25  Mar</t>
+        </is>
+      </c>
+      <c r="B236" s="39" t="inlineStr">
+        <is>
+          <t>03, 06, 09, 10, 18, 19, 24, 25, 26, 27, 33, 35, 37, 39, 48, 51, 53, 56, 65, 66</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +28 Pool hasta 2026-08-26
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -33420,7 +33420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B236"/>
+  <dimension ref="A1:B237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -36246,6 +36246,18 @@
       <c r="B236" s="39" t="inlineStr">
         <is>
           <t>03, 06, 09, 10, 18, 19, 24, 25, 26, 27, 33, 35, 37, 39, 48, 51, 53, 56, 65, 66</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-26  Mié</t>
+        </is>
+      </c>
+      <c r="B237" s="39" t="inlineStr">
+        <is>
+          <t>09, 13, 16, 17, 18, 19, 21, 22, 26, 29, 32, 37, 42, 45, 53, 61, 66, 69, 74, 76</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-08-27
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -33420,7 +33420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B237"/>
+  <dimension ref="A1:B238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -36258,6 +36258,18 @@
       <c r="B237" s="39" t="inlineStr">
         <is>
           <t>09, 13, 16, 17, 18, 19, 21, 22, 26, 29, 32, 37, 42, 45, 53, 61, 66, 69, 74, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-27  Jue</t>
+        </is>
+      </c>
+      <c r="B238" s="39" t="inlineStr">
+        <is>
+          <t>02, 13, 18, 22, 27, 28, 30, 33, 36, 37, 40, 46, 47, 51, 61, 62, 64, 66, 73, 74</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +125 Kino, + Pool hasta 2026-08-28
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -17616,7 +17616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B358"/>
+  <dimension ref="A1:B361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21906,6 +21906,42 @@
       <c r="A358" s="26" t="inlineStr">
         <is>
           <t>Total 2022: 355 sorteos  |  Generado 24/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="39" t="inlineStr">
+        <is>
+          <t>2022-01-15  Sáb</t>
+        </is>
+      </c>
+      <c r="B359" s="39" t="inlineStr">
+        <is>
+          <t>01, 04, 05, 08, 10, 12, 14, 15, 16, 20, 22, 29, 30, 31, 33, 37, 44, 47, 51, 61</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="39" t="inlineStr">
+        <is>
+          <t>2022-09-03  Sáb</t>
+        </is>
+      </c>
+      <c r="B360" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 07, 12, 16, 20, 27, 28, 31, 38, 44, 46, 47, 53, 56, 63, 65, 66, 68, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="39" t="inlineStr">
+        <is>
+          <t>2022-09-10  Sáb</t>
+        </is>
+      </c>
+      <c r="B361" s="39" t="inlineStr">
+        <is>
+          <t>02, 05, 07, 10, 14, 15, 22, 23, 24, 25, 26, 34, 40, 41, 42, 50, 56, 57, 60, 62</t>
         </is>
       </c>
     </row>
@@ -21924,7 +21960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B238"/>
+  <dimension ref="A1:B358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -24774,6 +24810,1446 @@
       <c r="A238" s="26" t="inlineStr">
         <is>
           <t>Total 2023: 235 sorteos  |  Generado 24/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="39" t="inlineStr">
+        <is>
+          <t>2023-03-30  Jue</t>
+        </is>
+      </c>
+      <c r="B239" s="39" t="inlineStr">
+        <is>
+          <t>01, 06, 08, 10, 12, 27, 28, 29, 30, 35, 49, 52, 54, 59, 60, 61, 68, 71, 74, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="39" t="inlineStr">
+        <is>
+          <t>2023-03-31  Vie</t>
+        </is>
+      </c>
+      <c r="B240" s="39" t="inlineStr">
+        <is>
+          <t>01, 08, 10, 16, 27, 29, 30, 31, 39, 40, 44, 51, 53, 54, 55, 59, 65, 73, 74, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-01  Sáb</t>
+        </is>
+      </c>
+      <c r="B241" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 05, 07, 13, 19, 21, 22, 25, 28, 32, 33, 35, 37, 46, 50, 53, 55, 72, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-02  Dom</t>
+        </is>
+      </c>
+      <c r="B242" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 09, 16, 17, 18, 23, 27, 30, 36, 41, 47, 49, 55, 64, 73, 74, 76, 77, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-03  Lun</t>
+        </is>
+      </c>
+      <c r="B243" s="39" t="inlineStr">
+        <is>
+          <t>03, 06, 09, 14, 15, 18, 19, 20, 24, 33, 36, 43, 48, 50, 52, 54, 61, 70, 73, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-04  Mar</t>
+        </is>
+      </c>
+      <c r="B244" s="39" t="inlineStr">
+        <is>
+          <t>04, 06, 09, 14, 15, 16, 19, 27, 32, 34, 39, 40, 47, 50, 51, 52, 53, 57, 60, 65</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-05  Mié</t>
+        </is>
+      </c>
+      <c r="B245" s="39" t="inlineStr">
+        <is>
+          <t>05, 06, 08, 10, 20, 22, 29, 32, 44, 48, 54, 55, 56, 60, 64, 69, 70, 71, 75, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-08  Sáb</t>
+        </is>
+      </c>
+      <c r="B246" s="39" t="inlineStr">
+        <is>
+          <t>08, 09, 11, 16, 19, 20, 22, 23, 32, 33, 41, 42, 45, 48, 53, 61, 67, 72, 74, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-09  Dom</t>
+        </is>
+      </c>
+      <c r="B247" s="39" t="inlineStr">
+        <is>
+          <t>06, 09, 15, 16, 17, 18, 19, 20, 29, 32, 33, 38, 39, 42, 54, 64, 68, 71, 73, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-10  Lun</t>
+        </is>
+      </c>
+      <c r="B248" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 04, 08, 10, 16, 29, 34, 42, 43, 47, 48, 50, 53, 54, 67, 69, 75, 76, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-11  Mar</t>
+        </is>
+      </c>
+      <c r="B249" s="39" t="inlineStr">
+        <is>
+          <t>03, 05, 11, 16, 24, 26, 27, 29, 33, 36, 37, 40, 41, 42, 50, 52, 54, 61, 62, 63</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-12  Mié</t>
+        </is>
+      </c>
+      <c r="B250" s="39" t="inlineStr">
+        <is>
+          <t>04, 05, 10, 12, 13, 14, 28, 31, 38, 48, 52, 53, 58, 61, 65, 68, 72, 77, 79, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-13  Jue</t>
+        </is>
+      </c>
+      <c r="B251" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 05, 08, 10, 13, 22, 29, 33, 36, 43, 47, 48, 50, 53, 54, 65, 72, 73, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-14  Vie</t>
+        </is>
+      </c>
+      <c r="B252" s="39" t="inlineStr">
+        <is>
+          <t>11, 14, 19, 21, 24, 28, 33, 43, 49, 50, 55, 56, 59, 63, 66, 70, 72, 73, 75, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-15  Sáb</t>
+        </is>
+      </c>
+      <c r="B253" s="39" t="inlineStr">
+        <is>
+          <t>02, 08, 09, 10, 15, 19, 27, 30, 32, 37, 40, 45, 49, 52, 55, 61, 64, 67, 74, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-16  Dom</t>
+        </is>
+      </c>
+      <c r="B254" s="39" t="inlineStr">
+        <is>
+          <t>02, 07, 08, 16, 18, 23, 26, 31, 37, 43, 46, 47, 51, 55, 63, 65, 74, 75, 76, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-17  Lun</t>
+        </is>
+      </c>
+      <c r="B255" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 03, 08, 15, 17, 18, 20, 33, 35, 36, 37, 41, 43, 46, 62, 65, 66, 67, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-18  Mar</t>
+        </is>
+      </c>
+      <c r="B256" s="39" t="inlineStr">
+        <is>
+          <t>04, 07, 11, 13, 18, 21, 22, 23, 29, 36, 57, 58, 60, 61, 62, 65, 66, 72, 75, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-19  Mié</t>
+        </is>
+      </c>
+      <c r="B257" s="39" t="inlineStr">
+        <is>
+          <t>01, 10, 11, 13, 14, 16, 19, 26, 29, 31, 32, 37, 45, 48, 54, 61, 65, 66, 68, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-20  Jue</t>
+        </is>
+      </c>
+      <c r="B258" s="39" t="inlineStr">
+        <is>
+          <t>01, 06, 12, 17, 20, 27, 31, 39, 47, 51, 52, 58, 59, 60, 62, 64, 68, 70, 72, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-21  Vie</t>
+        </is>
+      </c>
+      <c r="B259" s="39" t="inlineStr">
+        <is>
+          <t>02, 07, 09, 21, 24, 25, 27, 28, 29, 33, 34, 36, 45, 46, 47, 49, 62, 68, 73, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-22  Sáb</t>
+        </is>
+      </c>
+      <c r="B260" s="39" t="inlineStr">
+        <is>
+          <t>03, 09, 10, 16, 18, 22, 23, 24, 32, 36, 37, 45, 46, 48, 55, 61, 71, 74, 76, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-23  Dom</t>
+        </is>
+      </c>
+      <c r="B261" s="39" t="inlineStr">
+        <is>
+          <t>01, 09, 13, 14, 17, 20, 23, 30, 31, 33, 36, 37, 39, 48, 50, 54, 69, 73, 74, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-24  Lun</t>
+        </is>
+      </c>
+      <c r="B262" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 10, 11, 24, 32, 41, 45, 46, 48, 50, 52, 55, 58, 60, 61, 63, 66, 74, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-25  Mar</t>
+        </is>
+      </c>
+      <c r="B263" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 04, 08, 19, 24, 25, 26, 27, 33, 41, 42, 46, 48, 50, 55, 60, 67, 71, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-26  Mié</t>
+        </is>
+      </c>
+      <c r="B264" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 05, 09, 19, 26, 32, 33, 35, 37, 43, 50, 54, 56, 62, 66, 71, 73, 78, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-27  Jue</t>
+        </is>
+      </c>
+      <c r="B265" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 05, 10, 17, 23, 27, 28, 34, 37, 38, 39, 43, 45, 52, 54, 60, 62, 63, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-28  Vie</t>
+        </is>
+      </c>
+      <c r="B266" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 04, 05, 08, 11, 13, 16, 17, 28, 29, 34, 50, 53, 60, 64, 73, 75, 76, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-29  Sáb</t>
+        </is>
+      </c>
+      <c r="B267" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 05, 13, 16, 29, 30, 31, 34, 35, 40, 44, 53, 56, 63, 65, 66, 71, 72, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="39" t="inlineStr">
+        <is>
+          <t>2023-04-30  Dom</t>
+        </is>
+      </c>
+      <c r="B268" s="39" t="inlineStr">
+        <is>
+          <t>04, 05, 07, 12, 22, 23, 25, 26, 27, 30, 32, 36, 39, 41, 42, 52, 67, 73, 74, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-01  Lun</t>
+        </is>
+      </c>
+      <c r="B269" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 04, 06, 08, 14, 31, 32, 36, 42, 43, 44, 52, 58, 63, 66, 69, 75, 77, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-02  Mar</t>
+        </is>
+      </c>
+      <c r="B270" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 04, 09, 12, 13, 15, 17, 23, 29, 31, 33, 34, 40, 48, 65, 69, 70, 76, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-03  Mié</t>
+        </is>
+      </c>
+      <c r="B271" s="39" t="inlineStr">
+        <is>
+          <t>03, 04, 12, 13, 16, 17, 22, 29, 32, 35, 36, 38, 42, 45, 47, 50, 62, 63, 65, 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-04  Jue</t>
+        </is>
+      </c>
+      <c r="B272" s="39" t="inlineStr">
+        <is>
+          <t>04, 11, 13, 15, 16, 18, 22, 28, 31, 35, 36, 39, 52, 56, 64, 69, 71, 72, 74, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-05  Vie</t>
+        </is>
+      </c>
+      <c r="B273" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 05, 12, 18, 20, 23, 31, 35, 37, 49, 54, 55, 61, 62, 63, 67, 68, 69, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-06  Sáb</t>
+        </is>
+      </c>
+      <c r="B274" s="39" t="inlineStr">
+        <is>
+          <t>06, 11, 14, 17, 21, 22, 25, 26, 38, 45, 47, 49, 55, 58, 69, 72, 74, 75, 76, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-07  Dom</t>
+        </is>
+      </c>
+      <c r="B275" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 05, 07, 11, 14, 18, 21, 25, 26, 27, 29, 35, 39, 40, 42, 45, 49, 68, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-08  Lun</t>
+        </is>
+      </c>
+      <c r="B276" s="39" t="inlineStr">
+        <is>
+          <t>02, 06, 08, 10, 19, 21, 23, 24, 35, 38, 43, 46, 50, 52, 53, 58, 65, 66, 67, 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-09  Mar</t>
+        </is>
+      </c>
+      <c r="B277" s="39" t="inlineStr">
+        <is>
+          <t>06, 07, 08, 09, 12, 29, 31, 36, 37, 38, 39, 43, 47, 61, 65, 66, 67, 68, 70, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-10  Mié</t>
+        </is>
+      </c>
+      <c r="B278" s="39" t="inlineStr">
+        <is>
+          <t>05, 07, 09, 10, 13, 20, 25, 40, 46, 49, 50, 51, 55, 63, 64, 66, 68, 72, 74, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-11  Jue</t>
+        </is>
+      </c>
+      <c r="B279" s="39" t="inlineStr">
+        <is>
+          <t>03, 04, 05, 07, 11, 16, 18, 20, 22, 25, 27, 36, 38, 47, 48, 49, 53, 63, 65, 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-12  Vie</t>
+        </is>
+      </c>
+      <c r="B280" s="39" t="inlineStr">
+        <is>
+          <t>09, 12, 18, 19, 22, 23, 25, 29, 32, 34, 35, 36, 39, 51, 55, 57, 72, 75, 76, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-13  Sáb</t>
+        </is>
+      </c>
+      <c r="B281" s="39" t="inlineStr">
+        <is>
+          <t>06, 09, 13, 14, 17, 18, 19, 21, 27, 31, 33, 36, 37, 40, 42, 44, 47, 61, 68, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-14  Dom</t>
+        </is>
+      </c>
+      <c r="B282" s="39" t="inlineStr">
+        <is>
+          <t>04, 09, 14, 18, 25, 26, 31, 33, 36, 40, 42, 43, 44, 45, 53, 59, 69, 70, 71, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-15  Lun</t>
+        </is>
+      </c>
+      <c r="B283" s="39" t="inlineStr">
+        <is>
+          <t>04, 07, 14, 15, 16, 21, 27, 28, 32, 41, 46, 49, 57, 60, 63, 65, 69, 73, 76, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-16  Mar</t>
+        </is>
+      </c>
+      <c r="B284" s="39" t="inlineStr">
+        <is>
+          <t>01, 05, 06, 14, 16, 17, 18, 19, 20, 23, 24, 27, 28, 30, 41, 51, 53, 55, 62, 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-17  Mié</t>
+        </is>
+      </c>
+      <c r="B285" s="39" t="inlineStr">
+        <is>
+          <t>03, 04, 09, 13, 17, 19, 21, 23, 27, 33, 36, 38, 42, 43, 51, 55, 57, 74, 76, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-18  Jue</t>
+        </is>
+      </c>
+      <c r="B286" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 05, 06, 11, 15, 18, 21, 25, 32, 34, 36, 40, 41, 61, 62, 64, 65, 76, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-19  Vie</t>
+        </is>
+      </c>
+      <c r="B287" s="39" t="inlineStr">
+        <is>
+          <t>04, 08, 09, 13, 16, 19, 20, 22, 27, 36, 41, 51, 52, 58, 64, 66, 67, 68, 72, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-20  Sáb</t>
+        </is>
+      </c>
+      <c r="B288" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 05, 07, 15, 18, 20, 23, 26, 27, 34, 35, 37, 38, 44, 47, 48, 52, 59, 61</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-21  Dom</t>
+        </is>
+      </c>
+      <c r="B289" s="39" t="inlineStr">
+        <is>
+          <t>07, 11, 14, 16, 21, 22, 24, 25, 37, 40, 41, 42, 50, 53, 55, 57, 61, 63, 64, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-22  Lun</t>
+        </is>
+      </c>
+      <c r="B290" s="39" t="inlineStr">
+        <is>
+          <t>03, 07, 09, 10, 13, 14, 22, 23, 25, 26, 35, 36, 38, 39, 45, 47, 50, 60, 61, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-23  Mar</t>
+        </is>
+      </c>
+      <c r="B291" s="39" t="inlineStr">
+        <is>
+          <t>08, 09, 16, 20, 21, 23, 26, 27, 29, 40, 55, 57, 58, 59, 64, 65, 66, 68, 78, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-24  Mié</t>
+        </is>
+      </c>
+      <c r="B292" s="39" t="inlineStr">
+        <is>
+          <t>04, 13, 15, 17, 18, 21, 23, 24, 25, 43, 44, 46, 47, 52, 54, 55, 56, 59, 73, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-25  Jue</t>
+        </is>
+      </c>
+      <c r="B293" s="39" t="inlineStr">
+        <is>
+          <t>02, 14, 18, 20, 25, 27, 29, 30, 32, 33, 34, 47, 48, 49, 56, 61, 62, 67, 68, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-26  Vie</t>
+        </is>
+      </c>
+      <c r="B294" s="39" t="inlineStr">
+        <is>
+          <t>05, 06, 16, 18, 19, 22, 23, 26, 29, 31, 32, 37, 39, 41, 43, 47, 52, 53, 75, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-27  Sáb</t>
+        </is>
+      </c>
+      <c r="B295" s="39" t="inlineStr">
+        <is>
+          <t>01, 06, 12, 13, 21, 22, 25, 27, 31, 33, 35, 38, 44, 47, 49, 61, 64, 65, 69, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-28  Dom</t>
+        </is>
+      </c>
+      <c r="B296" s="39" t="inlineStr">
+        <is>
+          <t>02, 14, 16, 17, 28, 31, 33, 39, 44, 47, 49, 53, 55, 57, 61, 66, 69, 70, 72, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-29  Lun</t>
+        </is>
+      </c>
+      <c r="B297" s="39" t="inlineStr">
+        <is>
+          <t>04, 07, 08, 11, 18, 20, 22, 25, 27, 28, 29, 39, 40, 41, 49, 60, 62, 64, 66, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-30  Mar</t>
+        </is>
+      </c>
+      <c r="B298" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 09, 16, 27, 28, 30, 38, 39, 46, 47, 54, 56, 61, 62, 64, 69, 71, 72, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="39" t="inlineStr">
+        <is>
+          <t>2023-05-31  Mié</t>
+        </is>
+      </c>
+      <c r="B299" s="39" t="inlineStr">
+        <is>
+          <t>03, 11, 13, 24, 25, 31, 33, 39, 44, 48, 49, 50, 54, 55, 61, 62, 70, 71, 72, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-01  Jue</t>
+        </is>
+      </c>
+      <c r="B300" s="39" t="inlineStr">
+        <is>
+          <t>01, 18, 25, 26, 27, 28, 36, 40, 41, 44, 46, 47, 49, 50, 52, 53, 60, 66, 73, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-02  Vie</t>
+        </is>
+      </c>
+      <c r="B301" s="39" t="inlineStr">
+        <is>
+          <t>02, 07, 10, 16, 18, 21, 24, 32, 35, 36, 40, 41, 51, 58, 60, 65, 67, 68, 69, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-03  Sáb</t>
+        </is>
+      </c>
+      <c r="B302" s="39" t="inlineStr">
+        <is>
+          <t>03, 05, 11, 13, 19, 26, 33, 36, 43, 46, 52, 54, 55, 57, 62, 65, 68, 70, 75, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-04  Dom</t>
+        </is>
+      </c>
+      <c r="B303" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 15, 21, 24, 28, 34, 38, 39, 41, 43, 57, 59, 61, 67, 68, 71, 73, 74, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-05  Lun</t>
+        </is>
+      </c>
+      <c r="B304" s="39" t="inlineStr">
+        <is>
+          <t>04, 05, 21, 23, 30, 33, 42, 47, 48, 50, 54, 60, 62, 69, 70, 71, 76, 77, 79, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-06  Mar</t>
+        </is>
+      </c>
+      <c r="B305" s="39" t="inlineStr">
+        <is>
+          <t>01, 06, 17, 19, 20, 33, 37, 39, 40, 43, 51, 52, 55, 58, 60, 66, 67, 70, 71, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-07  Mié</t>
+        </is>
+      </c>
+      <c r="B306" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 07, 12, 16, 17, 27, 32, 38, 44, 47, 50, 53, 56, 59, 64, 65, 71, 72, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-08  Jue</t>
+        </is>
+      </c>
+      <c r="B307" s="39" t="inlineStr">
+        <is>
+          <t>03, 05, 08, 12, 15, 17, 18, 26, 27, 37, 40, 41, 47, 57, 63, 65, 72, 73, 77, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-09  Vie</t>
+        </is>
+      </c>
+      <c r="B308" s="39" t="inlineStr">
+        <is>
+          <t>03, 06, 09, 10, 12, 39, 43, 45, 55, 56, 59, 61, 63, 65, 66, 67, 68, 70, 72, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-10  Sáb</t>
+        </is>
+      </c>
+      <c r="B309" s="39" t="inlineStr">
+        <is>
+          <t>02, 06, 10, 14, 15, 18, 19, 21, 28, 35, 45, 46, 52, 55, 56, 64, 69, 72, 75, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-11  Dom</t>
+        </is>
+      </c>
+      <c r="B310" s="39" t="inlineStr">
+        <is>
+          <t>01, 11, 12, 14, 16, 20, 22, 30, 31, 34, 39, 40, 43, 44, 48, 56, 59, 60, 69, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-12  Lun</t>
+        </is>
+      </c>
+      <c r="B311" s="39" t="inlineStr">
+        <is>
+          <t>03, 05, 09, 12, 20, 21, 32, 33, 34, 37, 41, 46, 48, 51, 59, 67, 69, 71, 73, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-13  Mar</t>
+        </is>
+      </c>
+      <c r="B312" s="39" t="inlineStr">
+        <is>
+          <t>01, 04, 07, 13, 15, 19, 23, 24, 42, 43, 46, 52, 53, 60, 61, 64, 69, 70, 72, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-14  Mié</t>
+        </is>
+      </c>
+      <c r="B313" s="39" t="inlineStr">
+        <is>
+          <t>01, 06, 14, 15, 18, 20, 23, 26, 30, 33, 39, 40, 49, 50, 56, 57, 61, 66, 73, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-15  Jue</t>
+        </is>
+      </c>
+      <c r="B314" s="39" t="inlineStr">
+        <is>
+          <t>13, 15, 19, 21, 23, 25, 27, 30, 32, 36, 37, 43, 47, 49, 56, 59, 65, 67, 68, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-16  Vie</t>
+        </is>
+      </c>
+      <c r="B315" s="39" t="inlineStr">
+        <is>
+          <t>02, 06, 08, 11, 14, 16, 17, 21, 37, 44, 45, 48, 51, 55, 56, 59, 60, 67, 70, 71</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-17  Sáb</t>
+        </is>
+      </c>
+      <c r="B316" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 08, 09, 11, 15, 17, 29, 36, 37, 44, 47, 50, 52, 59, 60, 67, 72, 73, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-18  Dom</t>
+        </is>
+      </c>
+      <c r="B317" s="39" t="inlineStr">
+        <is>
+          <t>04, 11, 12, 13, 18, 20, 21, 28, 29, 36, 47, 49, 55, 57, 61, 64, 68, 71, 73, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-19  Lun</t>
+        </is>
+      </c>
+      <c r="B318" s="39" t="inlineStr">
+        <is>
+          <t>01, 09, 11, 15, 16, 17, 19, 24, 25, 36, 39, 44, 53, 56, 62, 69, 71, 72, 76, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-20  Mar</t>
+        </is>
+      </c>
+      <c r="B319" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 12, 16, 19, 20, 25, 27, 30, 34, 35, 41, 45, 47, 53, 64, 67, 69, 74, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-21  Mié</t>
+        </is>
+      </c>
+      <c r="B320" s="39" t="inlineStr">
+        <is>
+          <t>07, 16, 17, 20, 21, 31, 32, 35, 37, 39, 40, 41, 47, 48, 52, 61, 62, 64, 65, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-22  Jue</t>
+        </is>
+      </c>
+      <c r="B321" s="39" t="inlineStr">
+        <is>
+          <t>01, 04, 07, 08, 09, 16, 19, 21, 22, 27, 29, 36, 37, 45, 52, 55, 58, 63, 71, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-23  Vie</t>
+        </is>
+      </c>
+      <c r="B322" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 05, 06, 14, 23, 29, 31, 32, 33, 34, 35, 36, 45, 48, 49, 55, 70, 72, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-24  Sáb</t>
+        </is>
+      </c>
+      <c r="B323" s="39" t="inlineStr">
+        <is>
+          <t>02, 05, 12, 13, 22, 24, 30, 31, 35, 37, 38, 41, 42, 43, 48, 53, 54, 64, 72, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-25  Dom</t>
+        </is>
+      </c>
+      <c r="B324" s="39" t="inlineStr">
+        <is>
+          <t>02, 07, 08, 10, 14, 16, 23, 25, 26, 31, 33, 36, 37, 47, 53, 56, 58, 67, 75, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-26  Lun</t>
+        </is>
+      </c>
+      <c r="B325" s="39" t="inlineStr">
+        <is>
+          <t>03, 09, 10, 12, 13, 14, 21, 25, 26, 27, 39, 40, 41, 42, 43, 49, 55, 57, 73, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-27  Mar</t>
+        </is>
+      </c>
+      <c r="B326" s="39" t="inlineStr">
+        <is>
+          <t>02, 07, 13, 16, 17, 20, 22, 27, 28, 32, 38, 41, 44, 47, 55, 59, 63, 64, 74, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-28  Mié</t>
+        </is>
+      </c>
+      <c r="B327" s="39" t="inlineStr">
+        <is>
+          <t>02, 10, 12, 13, 14, 16, 18, 27, 28, 29, 31, 32, 34, 35, 49, 51, 52, 55, 58, 63</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-29  Jue</t>
+        </is>
+      </c>
+      <c r="B328" s="39" t="inlineStr">
+        <is>
+          <t>04, 08, 10, 11, 12, 17, 23, 29, 34, 39, 43, 45, 49, 58, 59, 64, 67, 69, 70, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="39" t="inlineStr">
+        <is>
+          <t>2023-06-30  Vie</t>
+        </is>
+      </c>
+      <c r="B329" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 13, 20, 24, 26, 27, 30, 33, 35, 41, 42, 43, 45, 48, 57, 62, 68, 74, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-01  Sáb</t>
+        </is>
+      </c>
+      <c r="B330" s="39" t="inlineStr">
+        <is>
+          <t>01, 07, 10, 13, 15, 20, 27, 32, 37, 39, 44, 47, 49, 56, 58, 59, 64, 66, 74, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-02  Dom</t>
+        </is>
+      </c>
+      <c r="B331" s="39" t="inlineStr">
+        <is>
+          <t>02, 13, 14, 16, 17, 18, 20, 22, 27, 36, 38, 39, 40, 49, 55, 64, 68, 74, 75, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-03  Lun</t>
+        </is>
+      </c>
+      <c r="B332" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 07, 13, 22, 23, 26, 28, 30, 31, 34, 48, 53, 55, 59, 63, 66, 69, 71, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-04  Mar</t>
+        </is>
+      </c>
+      <c r="B333" s="39" t="inlineStr">
+        <is>
+          <t>03, 04, 12, 14, 20, 30, 32, 39, 41, 43, 44, 46, 47, 49, 50, 51, 60, 64, 65, 66</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-05  Mié</t>
+        </is>
+      </c>
+      <c r="B334" s="39" t="inlineStr">
+        <is>
+          <t>01, 05, 08, 11, 12, 13, 18, 29, 33, 38, 41, 43, 45, 46, 51, 54, 69, 70, 71, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-06  Jue</t>
+        </is>
+      </c>
+      <c r="B335" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 04, 06, 10, 23, 24, 30, 35, 38, 41, 43, 47, 50, 56, 59, 65, 70, 71, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-07  Vie</t>
+        </is>
+      </c>
+      <c r="B336" s="39" t="inlineStr">
+        <is>
+          <t>07, 16, 20, 21, 22, 25, 33, 34, 37, 42, 48, 49, 54, 60, 61, 63, 64, 70, 72, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-08  Sáb</t>
+        </is>
+      </c>
+      <c r="B337" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 08, 15, 17, 26, 29, 31, 39, 40, 43, 54, 59, 62, 64, 65, 66, 72, 77, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-09  Dom</t>
+        </is>
+      </c>
+      <c r="B338" s="39" t="inlineStr">
+        <is>
+          <t>03, 07, 09, 10, 14, 17, 22, 32, 36, 37, 40, 42, 43, 46, 49, 51, 57, 62, 68, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-10  Lun</t>
+        </is>
+      </c>
+      <c r="B339" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 04, 10, 16, 17, 18, 21, 22, 30, 33, 35, 38, 50, 59, 60, 61, 65, 67, 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-11  Mar</t>
+        </is>
+      </c>
+      <c r="B340" s="39" t="inlineStr">
+        <is>
+          <t>03, 05, 10, 11, 15, 22, 26, 31, 36, 42, 45, 49, 50, 56, 57, 60, 67, 75, 78, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-12  Mié</t>
+        </is>
+      </c>
+      <c r="B341" s="39" t="inlineStr">
+        <is>
+          <t>12, 15, 18, 26, 36, 38, 40, 43, 45, 46, 54, 55, 58, 61, 67, 68, 72, 73, 78, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-13  Jue</t>
+        </is>
+      </c>
+      <c r="B342" s="39" t="inlineStr">
+        <is>
+          <t>02, 09, 12, 13, 16, 17, 19, 27, 30, 31, 38, 41, 43, 44, 48, 53, 54, 56, 57, 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-14  Vie</t>
+        </is>
+      </c>
+      <c r="B343" s="39" t="inlineStr">
+        <is>
+          <t>14, 17, 23, 28, 30, 36, 38, 42, 43, 45, 46, 48, 60, 62, 64, 68, 72, 73, 79, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-15  Sáb</t>
+        </is>
+      </c>
+      <c r="B344" s="39" t="inlineStr">
+        <is>
+          <t>03, 12, 15, 16, 19, 20, 26, 35, 37, 39, 42, 52, 54, 56, 57, 58, 61, 64, 66, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-16  Dom</t>
+        </is>
+      </c>
+      <c r="B345" s="39" t="inlineStr">
+        <is>
+          <t>07, 08, 16, 17, 20, 21, 25, 26, 34, 38, 42, 46, 49, 59, 64, 65, 72, 73, 74, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-17  Lun</t>
+        </is>
+      </c>
+      <c r="B346" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 17, 19, 29, 30, 33, 38, 42, 47, 48, 49, 52, 53, 56, 68, 72, 73, 78, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-18  Mar</t>
+        </is>
+      </c>
+      <c r="B347" s="39" t="inlineStr">
+        <is>
+          <t>07, 08, 18, 30, 33, 39, 42, 45, 47, 51, 55, 56, 57, 60, 65, 67, 68, 70, 74, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-19  Mié</t>
+        </is>
+      </c>
+      <c r="B348" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 07, 16, 18, 19, 22, 23, 24, 32, 37, 38, 45, 57, 59, 61, 67, 70, 73, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-20  Jue</t>
+        </is>
+      </c>
+      <c r="B349" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 04, 08, 12, 16, 20, 22, 24, 28, 32, 38, 40, 43, 51, 53, 54, 55, 61, 67</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-21  Vie</t>
+        </is>
+      </c>
+      <c r="B350" s="39" t="inlineStr">
+        <is>
+          <t>03, 04, 05, 20, 21, 22, 24, 39, 43, 44, 45, 47, 53, 55, 56, 57, 58, 61, 64, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-22  Sáb</t>
+        </is>
+      </c>
+      <c r="B351" s="39" t="inlineStr">
+        <is>
+          <t>01, 06, 13, 16, 18, 22, 27, 34, 36, 39, 45, 58, 60, 62, 67, 71, 73, 76, 77, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-23  Dom</t>
+        </is>
+      </c>
+      <c r="B352" s="39" t="inlineStr">
+        <is>
+          <t>03, 08, 11, 15, 21, 23, 24, 31, 35, 37, 38, 39, 43, 47, 48, 49, 54, 55, 64, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-24  Lun</t>
+        </is>
+      </c>
+      <c r="B353" s="39" t="inlineStr">
+        <is>
+          <t>02, 05, 07, 16, 17, 19, 24, 28, 33, 39, 43, 44, 48, 52, 59, 61, 65, 70, 75, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-25  Mar</t>
+        </is>
+      </c>
+      <c r="B354" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 05, 08, 14, 15, 17, 23, 24, 25, 39, 41, 50, 55, 60, 61, 62, 66, 73, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-26  Mié</t>
+        </is>
+      </c>
+      <c r="B355" s="39" t="inlineStr">
+        <is>
+          <t>03, 08, 14, 20, 26, 27, 28, 30, 35, 37, 45, 48, 49, 56, 57, 62, 65, 67, 77, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-27  Jue</t>
+        </is>
+      </c>
+      <c r="B356" s="39" t="inlineStr">
+        <is>
+          <t>04, 10, 16, 21, 26, 27, 31, 34, 35, 43, 50, 55, 58, 60, 61, 66, 68, 70, 71, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-28  Vie</t>
+        </is>
+      </c>
+      <c r="B357" s="39" t="inlineStr">
+        <is>
+          <t>03, 09, 10, 11, 22, 25, 28, 29, 37, 38, 40, 44, 47, 58, 63, 64, 69, 73, 74, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="39" t="inlineStr">
+        <is>
+          <t>2023-07-29  Sáb</t>
+        </is>
+      </c>
+      <c r="B358" s="39" t="inlineStr">
+        <is>
+          <t>01, 03, 04, 05, 15, 21, 29, 31, 35, 53, 55, 59, 60, 63, 67, 69, 70, 71, 76, 77</t>
         </is>
       </c>
     </row>
@@ -33420,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B238"/>
+  <dimension ref="A1:B239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -36270,6 +37746,18 @@
       <c r="B238" s="39" t="inlineStr">
         <is>
           <t>02, 13, 18, 22, 27, 28, 30, 33, 36, 37, 40, 46, 47, 51, 61, 62, 64, 66, 73, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-28  Vie</t>
+        </is>
+      </c>
+      <c r="B239" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 04, 06, 07, 19, 28, 38, 41, 43, 46, 52, 55, 59, 64, 66, 69, 73, 74, 76</t>
         </is>
       </c>
     </row>
@@ -60240,7 +61728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B368"/>
+  <dimension ref="A1:B369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -64650,6 +66138,18 @@
       <c r="A368" s="26" t="inlineStr">
         <is>
           <t>Total 2016: 365 sorteos  |  Generado 24/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="39" t="inlineStr">
+        <is>
+          <t>2016-02-08  Lun</t>
+        </is>
+      </c>
+      <c r="B369" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 07, 08, 10, 12, 23, 24, 32, 37, 39, 49, 53, 60, 62, 66, 67, 69, 73, 77</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-08-29
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B239"/>
+  <dimension ref="A1:B240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37758,6 +37758,18 @@
       <c r="B239" s="39" t="inlineStr">
         <is>
           <t>01, 02, 04, 06, 07, 19, 28, 38, 41, 43, 46, 52, 55, 59, 64, 66, 69, 73, 74, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-29  Sáb</t>
+        </is>
+      </c>
+      <c r="B240" s="39" t="inlineStr">
+        <is>
+          <t>12, 16, 22, 23, 25, 29, 32, 34, 36, 37, 40, 43, 47, 53, 56, 59, 67, 70, 72, 77</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +0 Pool hasta 2026-08-30
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B240"/>
+  <dimension ref="A1:B241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37770,6 +37770,18 @@
       <c r="B240" s="39" t="inlineStr">
         <is>
           <t>12, 16, 22, 23, 25, 29, 32, 34, 36, 37, 40, 43, 47, 53, 56, 59, 67, 70, 72, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-30  Dom</t>
+        </is>
+      </c>
+      <c r="B241" s="39" t="inlineStr">
+        <is>
+          <t>10, 20, 26, 27, 29, 30, 31, 34, 38, 46, 51, 52, 58, 59, 63, 70, 71, 75, 78, 79</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +0 Pool hasta 2026-08-31
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B241"/>
+  <dimension ref="A1:B242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37782,6 +37782,18 @@
       <c r="B241" s="39" t="inlineStr">
         <is>
           <t>10, 20, 26, 27, 29, 30, 31, 34, 38, 46, 51, 52, 58, 59, 63, 70, 71, 75, 78, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-31  Lun</t>
+        </is>
+      </c>
+      <c r="B242" s="39" t="inlineStr">
+        <is>
+          <t>06, 07, 10, 11, 15, 19, 24, 26, 31, 43, 46, 47, 52, 57, 65, 68, 69, 73, 74, 80</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +0 Pool hasta 2026-09-01
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B242"/>
+  <dimension ref="A1:B243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37794,6 +37794,18 @@
       <c r="B242" s="39" t="inlineStr">
         <is>
           <t>06, 07, 10, 11, 15, 19, 24, 26, 31, 43, 46, 47, 52, 57, 65, 68, 69, 73, 74, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-01  Mar</t>
+        </is>
+      </c>
+      <c r="B243" s="39" t="inlineStr">
+        <is>
+          <t>01, 10, 13, 18, 20, 22, 23, 25, 26, 27, 28, 33, 41, 49, 50, 54, 56, 62, 72, 79</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-02
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B243"/>
+  <dimension ref="A1:B244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37806,6 +37806,18 @@
       <c r="B243" s="39" t="inlineStr">
         <is>
           <t>01, 10, 13, 18, 20, 22, 23, 25, 26, 27, 28, 33, 41, 49, 50, 54, 56, 62, 72, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-02  Mié</t>
+        </is>
+      </c>
+      <c r="B244" s="39" t="inlineStr">
+        <is>
+          <t>02, 12, 13, 23, 27, 30, 37, 40, 47, 48, 49, 50, 53, 61, 62, 68, 71, 74, 77, 79</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +0 Pool hasta 2026-09-03
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B244"/>
+  <dimension ref="A1:B245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37818,6 +37818,18 @@
       <c r="B244" s="39" t="inlineStr">
         <is>
           <t>02, 12, 13, 23, 27, 30, 37, 40, 47, 48, 49, 50, 53, 61, 62, 68, 71, 74, 77, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-03  Jue</t>
+        </is>
+      </c>
+      <c r="B245" s="39" t="inlineStr">
+        <is>
+          <t>03, 14, 17, 22, 29, 30, 34, 35, 42, 47, 48, 57, 65, 66, 67, 68, 69, 70, 76, 77</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-04
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B245"/>
+  <dimension ref="A1:B246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37830,6 +37830,18 @@
       <c r="B245" s="39" t="inlineStr">
         <is>
           <t>03, 14, 17, 22, 29, 30, 34, 35, 42, 47, 48, 57, 65, 66, 67, 68, 69, 70, 76, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-04  Vie</t>
+        </is>
+      </c>
+      <c r="B246" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 06, 19, 24, 25, 29, 32, 33, 36, 37, 39, 41, 45, 46, 47, 53, 57, 63, 71</t>
         </is>
       </c>
     </row>

</xml_diff>